<commit_message>
Kalıp metraj detay çizimleri genişletildi — 7 SVG + mobil sayfa
- 01 tipik kat planı (perde/kolon/döşeme/kiriş)
- 02 temel/bodrum CAD planı (P109, BP1, BOŞLUK, T.Ü.K.)
- 03 +20,00 kalıp planı (D601/D602, K0601–K0604)
- 04 tam kot kesiti (−5,90 → +21,60)
- 05 kırık ölçü formülleri (örnek hesaplarla)
- 06 döşeme altı düşüm şeması
- 07 perde kalıp detay kesiti
- Poz bazlı metraj tablosu, Excel CAD eleman sayfası

Co-authored-by: barsokrr <barsokrr@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/metraj/Kalip_Metraj_Detay_Cizim.xlsx
+++ b/metraj/Kalip_Metraj_Detay_Cizim.xlsx
@@ -9,6 +9,7 @@
   <sheets>
     <sheet name="Metraj Detay" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Kat Kırılım" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="CAD Elemanlar" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -549,7 +550,7 @@
       </c>
       <c r="F4" s="3" t="inlineStr">
         <is>
-          <t>Σ kenar</t>
+          <t>150,5</t>
         </is>
       </c>
       <c r="G4" s="3" t="inlineStr">
@@ -567,7 +568,7 @@
       </c>
       <c r="J4" s="3" t="inlineStr">
         <is>
-          <t>Çevre 150,5×0,80</t>
+          <t>Çevre × h</t>
         </is>
       </c>
     </row>
@@ -663,7 +664,7 @@
       </c>
       <c r="J6" s="3" t="inlineStr">
         <is>
-          <t>150/35+180/30+60/60</t>
+          <t>13 adet</t>
         </is>
       </c>
     </row>
@@ -688,7 +689,7 @@
       </c>
       <c r="E7" s="3" t="inlineStr">
         <is>
-          <t>Perde ×4 aralık</t>
+          <t>Perde ×4</t>
         </is>
       </c>
       <c r="F7" s="3" t="inlineStr">
@@ -770,7 +771,7 @@
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>±0/+4/+8/+12/+16</t>
+          <t>5 kat</t>
         </is>
       </c>
       <c r="D9" s="3" t="inlineStr">
@@ -780,7 +781,7 @@
       </c>
       <c r="E9" s="3" t="inlineStr">
         <is>
-          <t>Alt kalıp ×5</t>
+          <t>Alt kalıp</t>
         </is>
       </c>
       <c r="F9" s="3" t="inlineStr">
@@ -851,7 +852,7 @@
       </c>
       <c r="J10" s="3" t="inlineStr">
         <is>
-          <t>Detay: KIRIS sayfası</t>
+          <t>H1 20/60 vb.</t>
         </is>
       </c>
     </row>
@@ -867,7 +868,7 @@
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:H1"/>
+    <mergeCell ref="A1:J1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1055,4 +1056,222 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E8"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="4" t="inlineStr">
+        <is>
+          <t>Plan</t>
+        </is>
+      </c>
+      <c r="B1" s="4" t="inlineStr">
+        <is>
+          <t>Etiket</t>
+        </is>
+      </c>
+      <c r="C1" s="4" t="inlineStr">
+        <is>
+          <t>Boyut</t>
+        </is>
+      </c>
+      <c r="D1" s="4" t="inlineStr">
+        <is>
+          <t>Tip</t>
+        </is>
+      </c>
+      <c r="E1" s="4" t="inlineStr">
+        <is>
+          <t>Not</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Temel</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>P109</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>30/160</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Perde</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Bodrum metraj</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Temel</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>P103</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>280/35</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Perde</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Temel</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>BP1</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>35/575</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Bodrum perde</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Temel</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>BOŞLUK</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>100/220</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Düşüm</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Metrajdan düşülür</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Temel</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>RD01</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>h=80</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Radye</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>T.Ü.K. −5,10</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Çatı +20</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>D601/D602</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>h=20</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Döşeme</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>650×650 iç</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Çatı +20</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>K0601–K0604</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>25/60</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Kiriş</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>